<commit_message>
Apply Saturday collection order update
</commit_message>
<xml_diff>
--- a/許可物件表_Git.xlsx
+++ b/許可物件表_Git.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="物件表" sheetId="1" r:id="R6aae28413acf4126"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属（行ってるとこコバ）" sheetId="2" r:id="R7f15bf14a59c4828"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表  (改定)" sheetId="3" r:id="R0a679ddf13e64776"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表  (uejii)" sheetId="4" r:id="R60a7d81011d447c6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表 " sheetId="5" r:id="R5b841beb61174cc8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日可燃収集表 (20250709)" sheetId="6" r:id="R0af5f3541a8e4d98"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="土曜日物件表 20250624" sheetId="7" r:id="R4bd314e69efb4416"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ガラ集物件（20250709）" sheetId="8" r:id="Rac6cccebf3a64f04"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="非表示物件" sheetId="9" r:id="Rd9fdbff360a44385"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="土曜日許可物件表（休出用）" sheetId="10" r:id="R1337011038634222"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="物件表" sheetId="1" r:id="R6502275b6b1544be"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属（行ってるとこコバ）" sheetId="2" r:id="R004a296d84704eeb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表  (改定)" sheetId="3" r:id="R28e70792fa594710"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表  (uejii)" sheetId="4" r:id="R537ae36f09244e60"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表 " sheetId="5" r:id="Ra67ac35f92bc4290"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日可燃収集表 (20250709)" sheetId="6" r:id="Rcbeaa0772bbc45bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="土曜日物件表 20250624" sheetId="7" r:id="Rb39f4562100640d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ガラ集物件（20250709）" sheetId="8" r:id="Ra60d768884f346c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="非表示物件" sheetId="9" r:id="R67742729c6db4a7f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="土曜日許可物件表（休出用）" sheetId="10" r:id="Rb04c7c0b201641a9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -13714,7 +13714,7 @@
       <x:c r="K298"/>
       <x:c r="L298"/>
       <x:c r="M298" t="str">
-        <x:v>外-</x:v>
+        <x:v>外-16</x:v>
       </x:c>
       <x:c r="N298"/>
       <x:c r="O298"/>

</xml_diff>

<commit_message>
Update Tuesday K collection order
</commit_message>
<xml_diff>
--- a/許可物件表_Git.xlsx
+++ b/許可物件表_Git.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="物件表" sheetId="1" r:id="R0349804f140f4042"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属（行ってるとこコバ）" sheetId="2" r:id="Rad2b095dee094a1f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表  (改定)" sheetId="3" r:id="R1d76e5b2d37b4251"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表  (uejii)" sheetId="4" r:id="Ra8bc4aa590184c6a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表 " sheetId="5" r:id="R049b42411e9d4ef4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日可燃収集表 (20250709)" sheetId="6" r:id="Ra835d2f2329640cd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="土曜日物件表 20250624" sheetId="7" r:id="Rde086491d7fa45c8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ガラ集物件（20250709）" sheetId="8" r:id="Rcef11ae0a546421f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="非表示物件" sheetId="9" r:id="Ra551e4ba175d44f6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="土曜日許可物件表（休出用）" sheetId="10" r:id="R433a993d0fc446fa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="物件表" sheetId="1" r:id="R9f94ddc77ac34784"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属（行ってるとこコバ）" sheetId="2" r:id="R9bc0a66d225c448e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表  (改定)" sheetId="3" r:id="R6c66fdc5cf774b77"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表  (uejii)" sheetId="4" r:id="R1f8101d8def34080"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表 " sheetId="5" r:id="R47a1cc45d6b24d39"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日可燃収集表 (20250709)" sheetId="6" r:id="R14792cc1f3014017"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="土曜日物件表 20250624" sheetId="7" r:id="Rf4cfdf8c11104ef2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ガラ集物件（20250709）" sheetId="8" r:id="R49a8a952c6344fa4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="非表示物件" sheetId="9" r:id="R25bb6dd509384679"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="土曜日許可物件表（休出用）" sheetId="10" r:id="R3897452f7978465a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3815,7 +3815,7 @@
       </x:c>
       <x:c r="H54"/>
       <x:c r="I54" t="str">
-        <x:v>K-</x:v>
+        <x:v>K-49</x:v>
       </x:c>
       <x:c r="J54"/>
       <x:c r="K54"/>
@@ -9597,7 +9597,7 @@
       </x:c>
       <x:c r="H194"/>
       <x:c r="I194" t="str">
-        <x:v>K-51</x:v>
+        <x:v>K-52</x:v>
       </x:c>
       <x:c r="J194"/>
       <x:c r="K194"/>
@@ -9637,7 +9637,7 @@
       </x:c>
       <x:c r="H195"/>
       <x:c r="I195" t="str">
-        <x:v>K-52</x:v>
+        <x:v>K-53</x:v>
       </x:c>
       <x:c r="J195"/>
       <x:c r="K195"/>
@@ -9717,7 +9717,7 @@
         <x:v>K-47</x:v>
       </x:c>
       <x:c r="I197" t="str">
-        <x:v>K-54</x:v>
+        <x:v>K-55</x:v>
       </x:c>
       <x:c r="J197" t="str">
         <x:v>K-28</x:v>
@@ -9765,7 +9765,7 @@
         <x:v>K-48</x:v>
       </x:c>
       <x:c r="I198" t="str">
-        <x:v>K-55</x:v>
+        <x:v>K-56</x:v>
       </x:c>
       <x:c r="J198" t="str">
         <x:v>K-29</x:v>
@@ -9967,7 +9967,7 @@
       </x:c>
       <x:c r="H203"/>
       <x:c r="I203" t="str">
-        <x:v>K-53</x:v>
+        <x:v>K-54</x:v>
       </x:c>
       <x:c r="J203"/>
       <x:c r="K203"/>
@@ -13651,7 +13651,7 @@
       </x:c>
       <x:c r="H295"/>
       <x:c r="I295" t="str">
-        <x:v>K-50</x:v>
+        <x:v>K-51</x:v>
       </x:c>
       <x:c r="J295"/>
       <x:c r="K295"/>

</xml_diff>

<commit_message>
Make metal collection order consecutive
</commit_message>
<xml_diff>
--- a/許可物件表_Git.xlsx
+++ b/許可物件表_Git.xlsx
@@ -9928,7 +9928,7 @@
       </c>
       <c r="P225" t="inlineStr">
         <is>
-          <t>金属-64</t>
+          <t>金属-63</t>
         </is>
       </c>
       <c r="R225" t="inlineStr">
@@ -10047,7 +10047,7 @@
       </c>
       <c r="P228" t="inlineStr">
         <is>
-          <t>金属-63</t>
+          <t>金属-62</t>
         </is>
       </c>
       <c r="R228" t="inlineStr">
@@ -10120,7 +10120,7 @@
       </c>
       <c r="P229" t="inlineStr">
         <is>
-          <t>金属-62</t>
+          <t>金属-61</t>
         </is>
       </c>
       <c r="R229" t="inlineStr">
@@ -10158,7 +10158,7 @@
       </c>
       <c r="P230" t="inlineStr">
         <is>
-          <t>金属-65</t>
+          <t>金属-64</t>
         </is>
       </c>
       <c r="T230" t="inlineStr">
@@ -10282,7 +10282,7 @@
       </c>
       <c r="P233" t="inlineStr">
         <is>
-          <t>金属-58</t>
+          <t>金属-57</t>
         </is>
       </c>
     </row>
@@ -10358,7 +10358,7 @@
       </c>
       <c r="P235" t="inlineStr">
         <is>
-          <t>金属-60</t>
+          <t>金属-59</t>
         </is>
       </c>
       <c r="R235" t="inlineStr">
@@ -10406,7 +10406,7 @@
       </c>
       <c r="P236" t="inlineStr">
         <is>
-          <t>金属-61</t>
+          <t>金属-60</t>
         </is>
       </c>
       <c r="R236" t="inlineStr">
@@ -10449,7 +10449,7 @@
       </c>
       <c r="P237" t="inlineStr">
         <is>
-          <t>金属-59</t>
+          <t>金属-58</t>
         </is>
       </c>
       <c r="R237" t="inlineStr">
@@ -10521,11 +10521,6 @@
       <c r="K239" t="inlineStr">
         <is>
           <t>K-34</t>
-        </is>
-      </c>
-      <c r="P239" t="inlineStr">
-        <is>
-          <t>金属-54</t>
         </is>
       </c>
       <c r="V239" t="inlineStr">

</xml_diff>

<commit_message>
Add Ichiko Haruta to metal collection order
</commit_message>
<xml_diff>
--- a/許可物件表_Git.xlsx
+++ b/許可物件表_Git.xlsx
@@ -9571,6 +9571,11 @@
           <t>K-6</t>
         </is>
       </c>
+      <c r="P215" t="inlineStr">
+        <is>
+          <t>金属-65</t>
+        </is>
+      </c>
     </row>
     <row r="216" ht="21" customHeight="1" s="10">
       <c r="A216" t="inlineStr">

</xml_diff>

<commit_message>
Mark Uchigane for metal collection
</commit_message>
<xml_diff>
--- a/許可物件表_Git.xlsx
+++ b/許可物件表_Git.xlsx
@@ -1793,6 +1793,11 @@
           <t>M-</t>
         </is>
       </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>金属-</t>
+        </is>
+      </c>
       <c r="Q24" t="inlineStr">
         <is>
           <t>段紙-5</t>

</xml_diff>

<commit_message>
Insert Uchigane into metal collection order
</commit_message>
<xml_diff>
--- a/許可物件表_Git.xlsx
+++ b/許可物件表_Git.xlsx
@@ -1752,7 +1752,7 @@
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>金属-6</t>
+          <t>金属-7</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
@@ -1795,7 +1795,7 @@
       </c>
       <c r="P24" t="inlineStr">
         <is>
-          <t>金属-</t>
+          <t>金属-6</t>
         </is>
       </c>
       <c r="Q24" t="inlineStr">
@@ -2463,7 +2463,7 @@
       </c>
       <c r="P40" t="inlineStr">
         <is>
-          <t>金属-19</t>
+          <t>金属-20</t>
         </is>
       </c>
       <c r="V40" t="inlineStr">
@@ -2681,7 +2681,7 @@
       </c>
       <c r="P46" t="inlineStr">
         <is>
-          <t>金属-20</t>
+          <t>金属-21</t>
         </is>
       </c>
       <c r="Q46" t="inlineStr">
@@ -3079,7 +3079,7 @@
       </c>
       <c r="P57" t="inlineStr">
         <is>
-          <t>金属-22</t>
+          <t>金属-23</t>
         </is>
       </c>
       <c r="V57" t="inlineStr">
@@ -3165,7 +3165,7 @@
       </c>
       <c r="P59" t="inlineStr">
         <is>
-          <t>金属-21</t>
+          <t>金属-22</t>
         </is>
       </c>
       <c r="V59" t="inlineStr">
@@ -3289,7 +3289,7 @@
       </c>
       <c r="P62" t="inlineStr">
         <is>
-          <t>金属-23</t>
+          <t>金属-24</t>
         </is>
       </c>
     </row>
@@ -3621,7 +3621,7 @@
       </c>
       <c r="P71" t="inlineStr">
         <is>
-          <t>金属-24</t>
+          <t>金属-25</t>
         </is>
       </c>
       <c r="R71" t="inlineStr">
@@ -3669,7 +3669,7 @@
       </c>
       <c r="P72" t="inlineStr">
         <is>
-          <t>金属-25</t>
+          <t>金属-26</t>
         </is>
       </c>
       <c r="T72" t="inlineStr">
@@ -4427,7 +4427,7 @@
       </c>
       <c r="P88" t="inlineStr">
         <is>
-          <t>金属-29</t>
+          <t>金属-30</t>
         </is>
       </c>
       <c r="R88" t="inlineStr">
@@ -4586,7 +4586,7 @@
       </c>
       <c r="P91" t="inlineStr">
         <is>
-          <t>金属-28</t>
+          <t>金属-29</t>
         </is>
       </c>
       <c r="R91" t="inlineStr">
@@ -4634,7 +4634,7 @@
       </c>
       <c r="P92" t="inlineStr">
         <is>
-          <t>金属-30</t>
+          <t>金属-31</t>
         </is>
       </c>
     </row>
@@ -4996,7 +4996,7 @@
       </c>
       <c r="P101" t="inlineStr">
         <is>
-          <t>金属-27</t>
+          <t>金属-28</t>
         </is>
       </c>
       <c r="Q101" t="inlineStr">
@@ -5120,7 +5120,7 @@
       </c>
       <c r="P104" t="inlineStr">
         <is>
-          <t>金属-26</t>
+          <t>金属-27</t>
         </is>
       </c>
       <c r="T104" t="inlineStr">
@@ -5436,7 +5436,7 @@
       </c>
       <c r="P111" t="inlineStr">
         <is>
-          <t>金属-31</t>
+          <t>金属-32</t>
         </is>
       </c>
       <c r="V111" t="inlineStr">
@@ -5542,7 +5542,7 @@
       </c>
       <c r="P113" t="inlineStr">
         <is>
-          <t>金属-33</t>
+          <t>金属-34</t>
         </is>
       </c>
       <c r="R113" t="inlineStr">
@@ -5600,7 +5600,7 @@
       </c>
       <c r="P114" t="inlineStr">
         <is>
-          <t>金属-32</t>
+          <t>金属-33</t>
         </is>
       </c>
       <c r="R114" t="inlineStr">
@@ -5668,7 +5668,7 @@
       </c>
       <c r="P115" t="inlineStr">
         <is>
-          <t>金属-34</t>
+          <t>金属-35</t>
         </is>
       </c>
       <c r="R115" t="inlineStr">
@@ -5711,7 +5711,7 @@
       </c>
       <c r="P116" t="inlineStr">
         <is>
-          <t>金属-35</t>
+          <t>金属-36</t>
         </is>
       </c>
     </row>
@@ -5891,7 +5891,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>金属-36</t>
+          <t>金属-37</t>
         </is>
       </c>
     </row>
@@ -6091,7 +6091,7 @@
       </c>
       <c r="P126" t="inlineStr">
         <is>
-          <t>金属-37</t>
+          <t>金属-38</t>
         </is>
       </c>
       <c r="R126" t="inlineStr">
@@ -6243,7 +6243,7 @@
       </c>
       <c r="P130" t="inlineStr">
         <is>
-          <t>金属-38</t>
+          <t>金属-39</t>
         </is>
       </c>
       <c r="T130" t="inlineStr">
@@ -6468,7 +6468,7 @@
       </c>
       <c r="P135" t="inlineStr">
         <is>
-          <t>金属-40</t>
+          <t>金属-41</t>
         </is>
       </c>
       <c r="Q135" t="inlineStr">
@@ -6549,7 +6549,7 @@
       </c>
       <c r="P137" t="inlineStr">
         <is>
-          <t>金属-41</t>
+          <t>金属-42</t>
         </is>
       </c>
     </row>
@@ -6658,7 +6658,7 @@
       </c>
       <c r="P140" t="inlineStr">
         <is>
-          <t>金属-42</t>
+          <t>金属-43</t>
         </is>
       </c>
     </row>
@@ -6706,7 +6706,7 @@
       </c>
       <c r="P141" t="inlineStr">
         <is>
-          <t>金属-43</t>
+          <t>金属-44</t>
         </is>
       </c>
     </row>
@@ -6744,7 +6744,7 @@
       </c>
       <c r="P142" t="inlineStr">
         <is>
-          <t>金属-39</t>
+          <t>金属-40</t>
         </is>
       </c>
     </row>
@@ -6830,7 +6830,7 @@
       </c>
       <c r="P144" t="inlineStr">
         <is>
-          <t>金属-44</t>
+          <t>金属-45</t>
         </is>
       </c>
       <c r="V144" t="inlineStr">
@@ -6878,7 +6878,7 @@
       </c>
       <c r="P145" t="inlineStr">
         <is>
-          <t>金属-45</t>
+          <t>金属-46</t>
         </is>
       </c>
     </row>
@@ -7025,7 +7025,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>金属-46</t>
+          <t>金属-47</t>
         </is>
       </c>
     </row>
@@ -7334,7 +7334,7 @@
       </c>
       <c r="P157" t="inlineStr">
         <is>
-          <t>金属-47</t>
+          <t>金属-48</t>
         </is>
       </c>
       <c r="R157" t="inlineStr">
@@ -7463,7 +7463,7 @@
       </c>
       <c r="P160" t="inlineStr">
         <is>
-          <t>金属-48</t>
+          <t>金属-49</t>
         </is>
       </c>
     </row>
@@ -7531,7 +7531,7 @@
       </c>
       <c r="P161" t="inlineStr">
         <is>
-          <t>金属-49</t>
+          <t>金属-50</t>
         </is>
       </c>
       <c r="Q161" t="inlineStr">
@@ -7683,7 +7683,7 @@
       </c>
       <c r="P165" t="inlineStr">
         <is>
-          <t>金属-50</t>
+          <t>金属-51</t>
         </is>
       </c>
       <c r="R165" t="inlineStr">
@@ -8005,7 +8005,7 @@
       </c>
       <c r="P174" t="inlineStr">
         <is>
-          <t>金属-52</t>
+          <t>金属-53</t>
         </is>
       </c>
     </row>
@@ -8134,7 +8134,7 @@
       </c>
       <c r="P177" t="inlineStr">
         <is>
-          <t>金属-51</t>
+          <t>金属-52</t>
         </is>
       </c>
       <c r="R177" t="inlineStr">
@@ -8309,7 +8309,7 @@
       </c>
       <c r="P182" t="inlineStr">
         <is>
-          <t>金属-53</t>
+          <t>金属-54</t>
         </is>
       </c>
     </row>
@@ -8347,7 +8347,7 @@
       </c>
       <c r="P183" t="inlineStr">
         <is>
-          <t>金属-54</t>
+          <t>金属-55</t>
         </is>
       </c>
     </row>
@@ -8380,7 +8380,7 @@
       </c>
       <c r="P184" t="inlineStr">
         <is>
-          <t>金属-55</t>
+          <t>金属-56</t>
         </is>
       </c>
     </row>
@@ -9578,7 +9578,7 @@
       </c>
       <c r="P215" t="inlineStr">
         <is>
-          <t>金属-65</t>
+          <t>金属-66</t>
         </is>
       </c>
     </row>
@@ -9938,7 +9938,7 @@
       </c>
       <c r="P225" t="inlineStr">
         <is>
-          <t>金属-63</t>
+          <t>金属-64</t>
         </is>
       </c>
       <c r="R225" t="inlineStr">
@@ -10057,7 +10057,7 @@
       </c>
       <c r="P228" t="inlineStr">
         <is>
-          <t>金属-62</t>
+          <t>金属-63</t>
         </is>
       </c>
       <c r="R228" t="inlineStr">
@@ -10130,7 +10130,7 @@
       </c>
       <c r="P229" t="inlineStr">
         <is>
-          <t>金属-61</t>
+          <t>金属-62</t>
         </is>
       </c>
       <c r="R229" t="inlineStr">
@@ -10168,7 +10168,7 @@
       </c>
       <c r="P230" t="inlineStr">
         <is>
-          <t>金属-64</t>
+          <t>金属-65</t>
         </is>
       </c>
       <c r="T230" t="inlineStr">
@@ -10292,7 +10292,7 @@
       </c>
       <c r="P233" t="inlineStr">
         <is>
-          <t>金属-57</t>
+          <t>金属-58</t>
         </is>
       </c>
     </row>
@@ -10368,7 +10368,7 @@
       </c>
       <c r="P235" t="inlineStr">
         <is>
-          <t>金属-59</t>
+          <t>金属-60</t>
         </is>
       </c>
       <c r="R235" t="inlineStr">
@@ -10416,7 +10416,7 @@
       </c>
       <c r="P236" t="inlineStr">
         <is>
-          <t>金属-60</t>
+          <t>金属-61</t>
         </is>
       </c>
       <c r="R236" t="inlineStr">
@@ -10459,7 +10459,7 @@
       </c>
       <c r="P237" t="inlineStr">
         <is>
-          <t>金属-58</t>
+          <t>金属-59</t>
         </is>
       </c>
       <c r="R237" t="inlineStr">
@@ -10573,7 +10573,7 @@
       </c>
       <c r="P240" t="inlineStr">
         <is>
-          <t>金属-56</t>
+          <t>金属-57</t>
         </is>
       </c>
       <c r="V240" t="inlineStr">
@@ -10816,7 +10816,7 @@
       </c>
       <c r="P246" t="inlineStr">
         <is>
-          <t>金属-14</t>
+          <t>金属-15</t>
         </is>
       </c>
       <c r="Q246" t="inlineStr">
@@ -10932,7 +10932,7 @@
       </c>
       <c r="P248" t="inlineStr">
         <is>
-          <t>金属-15</t>
+          <t>金属-16</t>
         </is>
       </c>
       <c r="Q248" t="inlineStr">
@@ -11008,7 +11008,7 @@
       </c>
       <c r="P250" t="inlineStr">
         <is>
-          <t>金属-17</t>
+          <t>金属-18</t>
         </is>
       </c>
     </row>
@@ -11046,7 +11046,7 @@
       </c>
       <c r="P251" t="inlineStr">
         <is>
-          <t>金属-18</t>
+          <t>金属-19</t>
         </is>
       </c>
     </row>
@@ -11089,7 +11089,7 @@
       </c>
       <c r="P252" t="inlineStr">
         <is>
-          <t>金属-16</t>
+          <t>金属-17</t>
         </is>
       </c>
       <c r="R252" t="inlineStr">
@@ -11216,7 +11216,7 @@
       </c>
       <c r="P256" t="inlineStr">
         <is>
-          <t>金属-13</t>
+          <t>金属-14</t>
         </is>
       </c>
     </row>
@@ -11282,7 +11282,7 @@
       </c>
       <c r="P258" t="inlineStr">
         <is>
-          <t>金属-12</t>
+          <t>金属-13</t>
         </is>
       </c>
       <c r="V258" t="inlineStr">
@@ -11434,7 +11434,7 @@
       </c>
       <c r="P262" t="inlineStr">
         <is>
-          <t>金属-11</t>
+          <t>金属-12</t>
         </is>
       </c>
       <c r="R262" t="inlineStr">
@@ -11520,7 +11520,7 @@
       </c>
       <c r="P264" t="inlineStr">
         <is>
-          <t>金属-8</t>
+          <t>金属-9</t>
         </is>
       </c>
       <c r="R264" t="inlineStr">
@@ -11806,7 +11806,7 @@
       </c>
       <c r="P271" t="inlineStr">
         <is>
-          <t>金属-7</t>
+          <t>金属-8</t>
         </is>
       </c>
       <c r="R271" t="inlineStr">
@@ -11968,7 +11968,7 @@
       </c>
       <c r="P275" t="inlineStr">
         <is>
-          <t>金属-10</t>
+          <t>金属-11</t>
         </is>
       </c>
       <c r="V275" t="inlineStr">
@@ -12110,7 +12110,7 @@
       </c>
       <c r="P279" t="inlineStr">
         <is>
-          <t>金属-9</t>
+          <t>金属-10</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update One Road property details
</commit_message>
<xml_diff>
--- a/許可物件表_Git.xlsx
+++ b/許可物件表_Git.xlsx
@@ -8560,12 +8560,22 @@
       </c>
       <c r="E189" t="inlineStr">
         <is>
-          <t>上野上柘植トラックセンター</t>
+          <t>One Road 上柘植トラックセンター</t>
         </is>
       </c>
       <c r="G189" t="inlineStr">
         <is>
           <t>45-8877</t>
+        </is>
+      </c>
+      <c r="J189" t="inlineStr">
+        <is>
+          <t>M-</t>
+        </is>
+      </c>
+      <c r="V189" t="inlineStr">
+        <is>
+          <t>第1第3水曜日</t>
         </is>
       </c>
     </row>

</xml_diff>